<commit_message>
Direct Write Excel for MIG CO2-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-01.xlsx
+++ b/FM-MN-07_MIG CO2-01.xlsx
@@ -1758,7 +1758,11 @@
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr"/>
-      <c r="H7" s="14" t="inlineStr"/>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="14" t="inlineStr"/>
       <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr"/>
@@ -1840,7 +1848,11 @@
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
       <c r="G8" s="14" t="inlineStr"/>
-      <c r="H8" s="14" t="inlineStr"/>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
       <c r="K8" s="14" t="inlineStr"/>
@@ -1881,7 +1893,11 @@
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
       <c r="G9" s="14" t="inlineStr"/>
-      <c r="H9" s="14" t="inlineStr"/>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
       <c r="K9" s="14" t="inlineStr"/>
@@ -1922,7 +1938,11 @@
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
       <c r="G10" s="14" t="inlineStr"/>
-      <c r="H10" s="14" t="inlineStr"/>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
       <c r="K10" s="14" t="inlineStr"/>
@@ -1963,7 +1983,11 @@
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
       <c r="G11" s="14" t="inlineStr"/>
-      <c r="H11" s="14" t="inlineStr"/>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
       <c r="K11" s="14" t="inlineStr"/>
@@ -2004,7 +2028,11 @@
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr"/>
-      <c r="H12" s="14" t="inlineStr"/>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
       <c r="K12" s="14" t="inlineStr"/>
@@ -2039,7 +2067,11 @@
       <c r="E13" s="27" t="inlineStr"/>
       <c r="F13" s="27" t="inlineStr"/>
       <c r="G13" s="27" t="inlineStr"/>
-      <c r="H13" s="27" t="inlineStr"/>
+      <c r="H13" s="39" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="I13" s="27" t="inlineStr"/>
       <c r="J13" s="27" t="inlineStr"/>
       <c r="K13" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MIG CO2-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-01.xlsx
+++ b/FM-MN-07_MIG CO2-01.xlsx
@@ -1763,7 +1763,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr"/>
       <c r="L6" s="14" t="inlineStr"/>
@@ -1808,7 +1812,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr"/>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr"/>
       <c r="L7" s="14" t="inlineStr"/>
@@ -1853,7 +1861,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr"/>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="14" t="inlineStr"/>
       <c r="K8" s="14" t="inlineStr"/>
       <c r="L8" s="14" t="inlineStr"/>
@@ -1898,7 +1910,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr"/>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="14" t="inlineStr"/>
       <c r="K9" s="14" t="inlineStr"/>
       <c r="L9" s="14" t="inlineStr"/>
@@ -1943,7 +1959,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr"/>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="14" t="inlineStr"/>
       <c r="K10" s="14" t="inlineStr"/>
       <c r="L10" s="14" t="inlineStr"/>
@@ -1988,7 +2008,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr"/>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="14" t="inlineStr"/>
       <c r="K11" s="14" t="inlineStr"/>
       <c r="L11" s="14" t="inlineStr"/>
@@ -2033,7 +2057,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="14" t="inlineStr"/>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="14" t="inlineStr"/>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="14" t="inlineStr"/>
@@ -2072,7 +2100,11 @@
           <t>อนุสรณ์  ชื่นแฉ่ง</t>
         </is>
       </c>
-      <c r="I13" s="27" t="inlineStr"/>
+      <c r="I13" s="39" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="J13" s="27" t="inlineStr"/>
       <c r="K13" s="27" t="inlineStr"/>
       <c r="L13" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MIG CO2-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-01.xlsx
+++ b/FM-MN-07_MIG CO2-01.xlsx
@@ -1768,7 +1768,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="14" t="inlineStr"/>
       <c r="L6" s="14" t="inlineStr"/>
       <c r="M6" s="14" t="inlineStr"/>
@@ -1817,7 +1821,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="14" t="inlineStr"/>
       <c r="L7" s="14" t="inlineStr"/>
       <c r="M7" s="14" t="inlineStr"/>
@@ -1866,7 +1874,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="14" t="inlineStr"/>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="14" t="inlineStr"/>
       <c r="L8" s="14" t="inlineStr"/>
       <c r="M8" s="14" t="inlineStr"/>
@@ -1915,7 +1927,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="14" t="inlineStr"/>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="14" t="inlineStr"/>
       <c r="L9" s="14" t="inlineStr"/>
       <c r="M9" s="14" t="inlineStr"/>
@@ -1964,7 +1980,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="14" t="inlineStr"/>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="14" t="inlineStr"/>
       <c r="L10" s="14" t="inlineStr"/>
       <c r="M10" s="14" t="inlineStr"/>
@@ -2013,7 +2033,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="14" t="inlineStr"/>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="14" t="inlineStr"/>
       <c r="L11" s="14" t="inlineStr"/>
       <c r="M11" s="14" t="inlineStr"/>
@@ -2062,7 +2086,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="14" t="inlineStr"/>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="14" t="inlineStr"/>
       <c r="M12" s="14" t="inlineStr"/>
@@ -2105,7 +2133,11 @@
           <t>อนุสรณ์  ชื่นแฉ่ง</t>
         </is>
       </c>
-      <c r="J13" s="27" t="inlineStr"/>
+      <c r="J13" s="39" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="K13" s="27" t="inlineStr"/>
       <c r="L13" s="27" t="inlineStr"/>
       <c r="M13" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MIG CO2-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-01.xlsx
+++ b/FM-MN-07_MIG CO2-01.xlsx
@@ -1774,7 +1774,11 @@
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr"/>
-      <c r="L6" s="14" t="inlineStr"/>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="14" t="inlineStr"/>
       <c r="N6" s="14" t="inlineStr"/>
       <c r="O6" s="14" t="inlineStr"/>
@@ -1827,7 +1831,11 @@
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr"/>
-      <c r="L7" s="14" t="inlineStr"/>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="14" t="inlineStr"/>
       <c r="N7" s="14" t="inlineStr"/>
       <c r="O7" s="14" t="inlineStr"/>
@@ -1880,7 +1888,11 @@
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr"/>
-      <c r="L8" s="14" t="inlineStr"/>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="14" t="inlineStr"/>
       <c r="N8" s="14" t="inlineStr"/>
       <c r="O8" s="14" t="inlineStr"/>
@@ -1933,7 +1945,11 @@
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr"/>
-      <c r="L9" s="14" t="inlineStr"/>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="14" t="inlineStr"/>
       <c r="N9" s="14" t="inlineStr"/>
       <c r="O9" s="14" t="inlineStr"/>
@@ -1986,7 +2002,11 @@
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr"/>
-      <c r="L10" s="14" t="inlineStr"/>
+      <c r="L10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="14" t="inlineStr"/>
       <c r="N10" s="14" t="inlineStr"/>
       <c r="O10" s="14" t="inlineStr"/>
@@ -2039,7 +2059,11 @@
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr"/>
-      <c r="L11" s="14" t="inlineStr"/>
+      <c r="L11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="14" t="inlineStr"/>
       <c r="N11" s="14" t="inlineStr"/>
       <c r="O11" s="14" t="inlineStr"/>
@@ -2092,7 +2116,11 @@
         </is>
       </c>
       <c r="K12" s="14" t="inlineStr"/>
-      <c r="L12" s="14" t="inlineStr"/>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="14" t="inlineStr"/>
       <c r="N12" s="14" t="inlineStr"/>
       <c r="O12" s="14" t="inlineStr"/>
@@ -2139,7 +2167,11 @@
         </is>
       </c>
       <c r="K13" s="27" t="inlineStr"/>
-      <c r="L13" s="27" t="inlineStr"/>
+      <c r="L13" s="39" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="M13" s="27" t="inlineStr"/>
       <c r="N13" s="27" t="inlineStr"/>
       <c r="O13" s="27" t="inlineStr"/>

</xml_diff>